<commit_message>
feat(planning): add multi-angle, image, design brief features + Brand Needs sheet
Adds four features surfaced by Matthew:
- F-053 Multiple positioning angles per avatar (Beta, P1)
- F-054 Image asset side-by-side comparison and tracking (GA, P1,
  conditional on asset-tracking decision)
- F-055 Design brief creation (Beta, P1)
- F-056 Image generation — 'coming soon' (Post-GA, P2)

Adds Brand Needs sheet seeded with InfinityVault as the first
validation case:
- N-001 Brand strategy doc for collector avatar (mapped to F-001,
  F-004..F-008, F-022, F-023)
- N-002 / N-002.1 / N-002.1.1 Assess images/videos, identify gaps,
  surface emotional-connection opportunities (mapped to F-006,
  F-007, F-054, F-055)

Each need's fulfilment_status derives from the status of mapped
features — same COUNTIFS pattern as the Phase Gate sheet.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/feature_status_tracker.xlsx
+++ b/docs/feature_status_tracker.xlsx
@@ -11,8 +11,9 @@
     <sheet name="Features" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Sub-features" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Phase Gate" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Risks" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Change Log" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Brand Needs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Risks" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Change Log" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -613,27 +614,27 @@
         </is>
       </c>
       <c r="B5" s="4">
-        <f>COUNTIF('Features'!$E$3:$E$57,"Alpha")</f>
+        <f>COUNTIF('Features'!$E$3:$E$61,"Alpha")</f>
         <v/>
       </c>
       <c r="C5" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Alpha",'Features'!$G$3:$G$57,"complete")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Alpha",'Features'!$G$3:$G$61,"complete")</f>
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Alpha",'Features'!$G$3:$G$57,"in_progress")+COUNTIFS('Features'!$E$3:$E$57,"Alpha",'Features'!$G$3:$G$57,"in_review")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Alpha",'Features'!$G$3:$G$61,"in_progress")+COUNTIFS('Features'!$E$3:$E$61,"Alpha",'Features'!$G$3:$G$61,"in_review")</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Alpha",'Features'!$G$3:$G$57,"blocked")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Alpha",'Features'!$G$3:$G$61,"blocked")</f>
         <v/>
       </c>
       <c r="F5" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Alpha",'Features'!$G$3:$G$57,"not_started")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Alpha",'Features'!$G$3:$G$61,"not_started")</f>
         <v/>
       </c>
       <c r="G5" s="5">
-        <f>IFERROR(ROUND(SUMIFS('Features'!$H$3:$H$57,'Features'!$E$3:$E$57,"Alpha")/(B5*100),3),0)</f>
+        <f>IFERROR(ROUND(SUMIFS('Features'!$H$3:$H$61,'Features'!$E$3:$E$61,"Alpha")/(B5*100),3),0)</f>
         <v/>
       </c>
       <c r="H5" s="4">
@@ -648,27 +649,27 @@
         </is>
       </c>
       <c r="B6" s="4">
-        <f>COUNTIF('Features'!$E$3:$E$57,"Beta")</f>
+        <f>COUNTIF('Features'!$E$3:$E$61,"Beta")</f>
         <v/>
       </c>
       <c r="C6" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Beta",'Features'!$G$3:$G$57,"complete")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Beta",'Features'!$G$3:$G$61,"complete")</f>
         <v/>
       </c>
       <c r="D6" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Beta",'Features'!$G$3:$G$57,"in_progress")+COUNTIFS('Features'!$E$3:$E$57,"Beta",'Features'!$G$3:$G$57,"in_review")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Beta",'Features'!$G$3:$G$61,"in_progress")+COUNTIFS('Features'!$E$3:$E$61,"Beta",'Features'!$G$3:$G$61,"in_review")</f>
         <v/>
       </c>
       <c r="E6" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Beta",'Features'!$G$3:$G$57,"blocked")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Beta",'Features'!$G$3:$G$61,"blocked")</f>
         <v/>
       </c>
       <c r="F6" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Beta",'Features'!$G$3:$G$57,"not_started")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Beta",'Features'!$G$3:$G$61,"not_started")</f>
         <v/>
       </c>
       <c r="G6" s="5">
-        <f>IFERROR(ROUND(SUMIFS('Features'!$H$3:$H$57,'Features'!$E$3:$E$57,"Beta")/(B6*100),3),0)</f>
+        <f>IFERROR(ROUND(SUMIFS('Features'!$H$3:$H$61,'Features'!$E$3:$E$61,"Beta")/(B6*100),3),0)</f>
         <v/>
       </c>
       <c r="H6" s="4">
@@ -683,27 +684,27 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>COUNTIF('Features'!$E$3:$E$57,"GA")</f>
+        <f>COUNTIF('Features'!$E$3:$E$61,"GA")</f>
         <v/>
       </c>
       <c r="C7" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"GA",'Features'!$G$3:$G$57,"complete")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"GA",'Features'!$G$3:$G$61,"complete")</f>
         <v/>
       </c>
       <c r="D7" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"GA",'Features'!$G$3:$G$57,"in_progress")+COUNTIFS('Features'!$E$3:$E$57,"GA",'Features'!$G$3:$G$57,"in_review")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"GA",'Features'!$G$3:$G$61,"in_progress")+COUNTIFS('Features'!$E$3:$E$61,"GA",'Features'!$G$3:$G$61,"in_review")</f>
         <v/>
       </c>
       <c r="E7" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"GA",'Features'!$G$3:$G$57,"blocked")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"GA",'Features'!$G$3:$G$61,"blocked")</f>
         <v/>
       </c>
       <c r="F7" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"GA",'Features'!$G$3:$G$57,"not_started")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"GA",'Features'!$G$3:$G$61,"not_started")</f>
         <v/>
       </c>
       <c r="G7" s="5">
-        <f>IFERROR(ROUND(SUMIFS('Features'!$H$3:$H$57,'Features'!$E$3:$E$57,"GA")/(B7*100),3),0)</f>
+        <f>IFERROR(ROUND(SUMIFS('Features'!$H$3:$H$61,'Features'!$E$3:$E$61,"GA")/(B7*100),3),0)</f>
         <v/>
       </c>
       <c r="H7" s="4">
@@ -718,27 +719,27 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>COUNTIF('Features'!$E$3:$E$57,"Post-GA")</f>
+        <f>COUNTIF('Features'!$E$3:$E$61,"Post-GA")</f>
         <v/>
       </c>
       <c r="C8" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Post-GA",'Features'!$G$3:$G$57,"complete")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Post-GA",'Features'!$G$3:$G$61,"complete")</f>
         <v/>
       </c>
       <c r="D8" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Post-GA",'Features'!$G$3:$G$57,"in_progress")+COUNTIFS('Features'!$E$3:$E$57,"Post-GA",'Features'!$G$3:$G$57,"in_review")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Post-GA",'Features'!$G$3:$G$61,"in_progress")+COUNTIFS('Features'!$E$3:$E$61,"Post-GA",'Features'!$G$3:$G$61,"in_review")</f>
         <v/>
       </c>
       <c r="E8" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Post-GA",'Features'!$G$3:$G$57,"blocked")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Post-GA",'Features'!$G$3:$G$61,"blocked")</f>
         <v/>
       </c>
       <c r="F8" s="4">
-        <f>COUNTIFS('Features'!$E$3:$E$57,"Post-GA",'Features'!$G$3:$G$57,"not_started")</f>
+        <f>COUNTIFS('Features'!$E$3:$E$61,"Post-GA",'Features'!$G$3:$G$61,"not_started")</f>
         <v/>
       </c>
       <c r="G8" s="5">
-        <f>IFERROR(ROUND(SUMIFS('Features'!$H$3:$H$57,'Features'!$E$3:$E$57,"Post-GA")/(B8*100),3),0)</f>
+        <f>IFERROR(ROUND(SUMIFS('Features'!$H$3:$H$61,'Features'!$E$3:$E$61,"Post-GA")/(B8*100),3),0)</f>
         <v/>
       </c>
       <c r="H8" s="4">
@@ -755,19 +756,19 @@
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="4">
-        <f>IFERROR(INDEX('Features'!A3:A57,MATCH("blocked",'Features'!$G$3:$G$57,0)),"None")</f>
+        <f>IFERROR(INDEX('Features'!A3:A61,MATCH("blocked",'Features'!$G$3:$G$61,0)),"None")</f>
         <v/>
       </c>
       <c r="B11" s="4">
-        <f>IFERROR(INDEX('Features'!B3:B57,MATCH("blocked",'Features'!$G$3:$G$57,0)),"None")</f>
+        <f>IFERROR(INDEX('Features'!B3:B61,MATCH("blocked",'Features'!$G$3:$G$61,0)),"None")</f>
         <v/>
       </c>
       <c r="C11" s="4">
-        <f>IFERROR(INDEX('Features'!E3:E57,MATCH("blocked",'Features'!$G$3:$G$57,0)),"")</f>
+        <f>IFERROR(INDEX('Features'!E3:E61,MATCH("blocked",'Features'!$G$3:$G$61,0)),"")</f>
         <v/>
       </c>
       <c r="D11" s="4">
-        <f>IFERROR(INDEX('Features'!I3:I57,MATCH("blocked",'Features'!$G$3:$G$57,0)),"")</f>
+        <f>IFERROR(INDEX('Features'!I3:I61,MATCH("blocked",'Features'!$G$3:$G$61,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -799,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4328,65 +4329,329 @@
     <row r="57" ht="42" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
+          <t>F-053</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Multiple positioning angles per avatar</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>avatar_builder</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Support multiple positioning / marketing angle variants for the same avatar — each angle has its own brand strategy doc / canvas section, but shares the underlying avatar.</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="4" t="inlineStr"/>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>Matthew</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>F-008,F-031</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="M57" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>Validates A/B angle testing for paying users. Each angle = a strategy variant tied to a canonical avatar. Surfaces in Coach mode and Export. OPEN: schema choice — separate canvases per angle vs angle-tagged sections within one canvas.</t>
+        </is>
+      </c>
+      <c r="O57" s="8" t="n">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="58" ht="42" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>F-054</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Image asset side-by-side comparison and tracking</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>asset_tracking</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Upload current image/video assets, view side-by-side, tag against avatar + angle, flag gaps and emotional-connection opportunities.</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>Conditional on F-028 (asset tracking decision)</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>Matthew</t>
+        </is>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>F-028,F-053</t>
+        </is>
+      </c>
+      <c r="L58" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="M58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" s="4" t="inlineStr">
+        <is>
+          <t>Extension of asset_tracking that goes beyond text. Anchored to InfinityVault need N-002 (assess images/videos, identify what's missing, surface emotional-connection opportunities). Requires image storage (Supabase Storage) and a comparison UI.</t>
+        </is>
+      </c>
+      <c r="O58" s="8" t="n">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="59" ht="42" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>F-055</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Design brief creation</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>create_mode</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Generate a design brief document from the Forensic Canvas + selected positioning angle. Output briefs creative work (image, video, packaging) for designers or agencies.</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="4" t="inlineStr"/>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>Matthew</t>
+        </is>
+      </c>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>F-008,F-053</t>
+        </is>
+      </c>
+      <c r="L59" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="M59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
+          <t>Sibling to F-020 (Amazon listing copy) and F-021 (Brand Voice Guide). Bridges the canvas to creative work. Required to make F-054 actionable (gap → brief → asset).</t>
+        </is>
+      </c>
+      <c r="O59" s="8" t="n">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="60" ht="42" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>F-056</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Image generation (coming soon)</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>create_mode</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Generate brand-aligned imagery directly from canvas + design brief. Marked 'coming soon' — Post-GA feature, not in active build.</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>Post-GA</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="H60" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="4" t="inlineStr"/>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>Matthew</t>
+        </is>
+      </c>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>F-055</t>
+        </is>
+      </c>
+      <c r="L60" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="M60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" s="4" t="inlineStr">
+        <is>
+          <t>Surfaced as 'coming soon' in UI (teaser). Closes the loop from canvas → design brief → generated imagery. No model choice locked in; defer until Post-GA stability work is done.</t>
+        </is>
+      </c>
+      <c r="O60" s="8" t="n">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="61" ht="42" customHeight="1">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
           <t>F-052</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>Lovable.dev vs existing codebase decision</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>infrastructure</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr">
         <is>
           <t>Architectural decision: build Gen 3 in Lovable.dev (per Trevor) or extend existing React codebase. Critical risk per Launch Roadmap.</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="E61" s="4" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="G57" s="4" t="inlineStr">
+      <c r="G61" s="4" t="inlineStr">
         <is>
           <t>blocked</t>
         </is>
       </c>
-      <c r="H57" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
+      <c r="H61" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
         <is>
           <t>Awaiting decision — flagged Critical in Risk Register</t>
         </is>
       </c>
-      <c r="J57" s="4" t="inlineStr">
+      <c r="J61" s="4" t="inlineStr">
         <is>
           <t>Matthew</t>
         </is>
       </c>
-      <c r="K57" s="4" t="inlineStr"/>
-      <c r="L57" s="4" t="n">
+      <c r="K61" s="4" t="inlineStr"/>
+      <c r="L61" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M57" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N57" s="4" t="inlineStr">
+      <c r="M61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
         <is>
           <t>DEFERRED DECISION. Trevor's Gen 3 Brief specifies Lovable; existing codebase is React + Supabase. Don't half-port. Default: extend existing repo until Matthew decides otherwise.</t>
         </is>
       </c>
-      <c r="O57" s="8" t="n">
+      <c r="O61" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4394,7 +4659,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <conditionalFormatting sqref="G3:G257">
+  <conditionalFormatting sqref="G3:G261">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"complete"</formula>
     </cfRule>
@@ -4412,16 +4677,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="C3:C257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
+    <dataValidation sqref="C3:C261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
       <formula1>"conversation,avatar_builder,canvas,create_mode,coach_mode,pay_gate,export,accounts,asset_tracking,feedback_loop,analytics,infrastructure,design_system"</formula1>
     </dataValidation>
-    <dataValidation sqref="E3:E257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
+    <dataValidation sqref="E3:E261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
       <formula1>"Alpha,Beta,GA,Post-GA"</formula1>
     </dataValidation>
-    <dataValidation sqref="F3:F257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
+    <dataValidation sqref="F3:F261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
       <formula1>"P0,P1,P2"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
+    <dataValidation sqref="G3:G261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
       <formula1>"not_started,in_progress,blocked,in_review,complete"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7466,7 +7731,7 @@
         </is>
       </c>
       <c r="E5" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-001",'Features'!$G$3:$G$57,"blocked")+COUNTIFS('Features'!$A$3:$A$57,"F-002",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-001",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-002",'Features'!$G$3:$G$57,"complete"))=2,"MET","OPEN — "&amp;(2-(COUNTIFS('Features'!$A$3:$A$57,"F-001",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-002",'Features'!$G$3:$G$57,"complete")))&amp;" of 2 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-002",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-002",'Features'!$G$3:$G$61,"complete"))=2,"MET","OPEN — "&amp;(2-(COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-002",'Features'!$G$3:$G$61,"complete")))&amp;" of 2 remaining"))</f>
         <v/>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -7497,7 +7762,7 @@
         </is>
       </c>
       <c r="E6" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-003",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-003",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-003",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -7528,7 +7793,7 @@
         </is>
       </c>
       <c r="E7" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-004",'Features'!$G$3:$G$57,"blocked")+COUNTIFS('Features'!$A$3:$A$57,"F-005",'Features'!$G$3:$G$57,"blocked")+COUNTIFS('Features'!$A$3:$A$57,"F-006",'Features'!$G$3:$G$57,"blocked")+COUNTIFS('Features'!$A$3:$A$57,"F-007",'Features'!$G$3:$G$57,"blocked")+COUNTIFS('Features'!$A$3:$A$57,"F-009",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-004",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-005",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-006",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-007",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-009",'Features'!$G$3:$G$57,"complete"))=5,"MET","OPEN — "&amp;(5-(COUNTIFS('Features'!$A$3:$A$57,"F-004",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-005",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-006",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-007",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-009",'Features'!$G$3:$G$57,"complete")))&amp;" of 5 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"complete"))=5,"MET","OPEN — "&amp;(5-(COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"complete")))&amp;" of 5 remaining"))</f>
         <v/>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -7559,7 +7824,7 @@
         </is>
       </c>
       <c r="E8" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-008",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-008",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-008",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -7590,7 +7855,7 @@
         </is>
       </c>
       <c r="E9" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-011",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-011",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-011",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-011",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-011",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-011",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -7621,7 +7886,7 @@
         </is>
       </c>
       <c r="E10" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-013",'Features'!$G$3:$G$57,"blocked")+COUNTIFS('Features'!$A$3:$A$57,"F-014",'Features'!$G$3:$G$57,"blocked")+COUNTIFS('Features'!$A$3:$A$57,"F-015",'Features'!$G$3:$G$57,"blocked")+COUNTIFS('Features'!$A$3:$A$57,"F-016",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-013",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-014",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-015",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-016",'Features'!$G$3:$G$57,"complete"))=4,"MET","OPEN — "&amp;(4-(COUNTIFS('Features'!$A$3:$A$57,"F-013",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-014",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-015",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-016",'Features'!$G$3:$G$57,"complete")))&amp;" of 4 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-013",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-014",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-015",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-016",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-013",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-014",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-015",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-016",'Features'!$G$3:$G$61,"complete"))=4,"MET","OPEN — "&amp;(4-(COUNTIFS('Features'!$A$3:$A$61,"F-013",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-014",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-015",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-016",'Features'!$G$3:$G$61,"complete")))&amp;" of 4 remaining"))</f>
         <v/>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -7652,7 +7917,7 @@
         </is>
       </c>
       <c r="E11" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-017",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-017",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-017",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-017",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-017",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-017",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F11" s="4" t="inlineStr"/>
@@ -7679,7 +7944,7 @@
         </is>
       </c>
       <c r="E12" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-018",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-018",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-018",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-018",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-018",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-018",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F12" s="4" t="inlineStr"/>
@@ -7706,7 +7971,7 @@
         </is>
       </c>
       <c r="E13" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-052",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-052",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-052",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-052",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-052",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-052",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -7737,7 +8002,7 @@
         </is>
       </c>
       <c r="E14" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-016",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-016",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-016",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-016",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-016",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-016",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -7768,7 +8033,7 @@
         </is>
       </c>
       <c r="E15" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-019",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-019",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-019",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-019",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-019",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-019",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -7799,7 +8064,7 @@
         </is>
       </c>
       <c r="E16" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-020",'Features'!$G$3:$G$57,"blocked")+COUNTIFS('Features'!$A$3:$A$57,"F-021",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-020",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-021",'Features'!$G$3:$G$57,"complete"))=2,"MET","OPEN — "&amp;(2-(COUNTIFS('Features'!$A$3:$A$57,"F-020",'Features'!$G$3:$G$57,"complete")+COUNTIFS('Features'!$A$3:$A$57,"F-021",'Features'!$G$3:$G$57,"complete")))&amp;" of 2 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"complete"))=2,"MET","OPEN — "&amp;(2-(COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"complete")))&amp;" of 2 remaining"))</f>
         <v/>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -7830,7 +8095,7 @@
         </is>
       </c>
       <c r="E17" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-022",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-022",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-022",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -7861,7 +8126,7 @@
         </is>
       </c>
       <c r="E18" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-023",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-023",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-023",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F18" s="4" t="inlineStr"/>
@@ -7888,7 +8153,7 @@
         </is>
       </c>
       <c r="E19" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-028",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-028",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-028",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -7919,7 +8184,7 @@
         </is>
       </c>
       <c r="E20" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-024",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-024",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-024",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-024",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-024",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-024",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
@@ -7946,7 +8211,7 @@
         </is>
       </c>
       <c r="E21" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-025",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-025",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-025",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-025",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-025",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-025",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F21" s="4" t="inlineStr"/>
@@ -7973,7 +8238,7 @@
         </is>
       </c>
       <c r="E22" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-027",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-027",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-027",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-027",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-027",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-027",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -8000,7 +8265,7 @@
         </is>
       </c>
       <c r="E23" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-031",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-031",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-031",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F23" s="4" t="inlineStr"/>
@@ -8027,7 +8292,7 @@
         </is>
       </c>
       <c r="E24" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-032",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-032",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-032",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-032",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-032",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-032",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -8054,7 +8319,7 @@
         </is>
       </c>
       <c r="E25" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-033",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-033",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-033",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-033",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-033",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-033",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F25" s="4" t="inlineStr"/>
@@ -8081,7 +8346,7 @@
         </is>
       </c>
       <c r="E26" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-034",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-034",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-034",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-034",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-034",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-034",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -8108,7 +8373,7 @@
         </is>
       </c>
       <c r="E27" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-037",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-037",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-037",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-037",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-037",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-037",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F27" s="4" t="inlineStr"/>
@@ -8135,7 +8400,7 @@
         </is>
       </c>
       <c r="E28" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-035",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-035",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-035",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-035",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-035",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-035",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -8162,7 +8427,7 @@
         </is>
       </c>
       <c r="E29" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-036",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-036",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-036",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-036",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-036",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-036",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F29" s="4" t="inlineStr"/>
@@ -8189,7 +8454,7 @@
         </is>
       </c>
       <c r="E30" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-034",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-034",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-034",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-034",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-034",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-034",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
@@ -8216,7 +8481,7 @@
         </is>
       </c>
       <c r="E31" s="4">
-        <f>IF((COUNTIFS('Features'!$A$3:$A$57,"F-038",'Features'!$G$3:$G$57,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$57,"F-038",'Features'!$G$3:$G$57,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$57,"F-038",'Features'!$G$3:$G$57,"complete")))&amp;" of 1 remaining"))</f>
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
         <v/>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -8251,6 +8516,213 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Brand Needs — concrete user needs mapped to features</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Anchors the feature inventory to real brand use cases. Each leaf need maps to one or more feature ids. fulfilment_status is derived: MET if all mapped features complete, BLOCKED if any are blocked, otherwise OPEN with count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>need_id</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>brand</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>need</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>mapped_features</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>fulfilment_status</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>N-001</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>InfinityVault</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Create brand strategy doc using the Coach for the 'collector' avatar</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>F-001,F-004,F-005,F-006,F-007,F-008,F-022,F-023</t>
+        </is>
+      </c>
+      <c r="E5" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"complete"))=8,"MET","OPEN — "&amp;(8-(COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"complete")))&amp;" of 8 remaining"))</f>
+        <v/>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>End-to-end happy path: Layer 1 conversation → Avatar Builder (collector) → Forensic Canvas → Coach refinement → Export. Validates the core product loop with a real brand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>N-002</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>InfinityVault</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Assess current set of images and videos</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>F-054</t>
+        </is>
+      </c>
+      <c r="E6" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
+        <v/>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Top-level need under which the gap-identification and emotional-connection needs sit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>N-002.1</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>InfinityVault</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Identify what's missing in the current image/video set</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>F-054</t>
+        </is>
+      </c>
+      <c r="E7" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete"))=1,"MET","OPEN — "&amp;(1-(COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")))&amp;" of 1 remaining"))</f>
+        <v/>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Gap analysis on visual assets — requires side-by-side comparison + tagging against the canvas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>N-002.1.1</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>InfinityVault</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Surface opportunities to improve emotional connection with the customer</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>F-006,F-007,F-054,F-055</t>
+        </is>
+      </c>
+      <c r="E8" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete"))=4,"MET","OPEN — "&amp;(4-(COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")))&amp;" of 4 remaining"))</f>
+        <v/>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Connects Emotional Journey Mapping (Avatar Builder Sec 3) + Voice of Customer (Sec 4) to the asset gaps surfaced by F-054, with design briefs (F-055) closing the loop into action.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E5:E8">
+    <cfRule type="expression" priority="1" dxfId="2">
+      <formula>E5="MET"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>ISNUMBER(SEARCH("BLOCKED",E5))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>ISNUMBER(SEARCH("OPEN",E5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8985,13 +9457,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9051,6 +9523,28 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Matthew (via Claude Code)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Added F-053..F-056 + Brand Needs sheet</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Captured multi-angle, image comparison, design brief, and (post-GA) image generation features. Added Brand Needs sheet seeded with InfinityVault as the first validation case.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
fix(planning): correct status for brand strategy doc + PDF export
I had the workbook wrong on three features that are substantially shipped:

- F-008 Forensic Canvas synthesis: was not_started 0% → now
  in_review 80%. The generate-brand-strategy-document edge function
  (1164 LoC, pgvector RAG, Haiku, client-side orchestration) IS this
  in current code. Remaining: explicit 'Strategic Entry Point'
  Trigger Moment callout + Draft↔Forensic toggle.
- F-023 Export PDF and Word: was not_started 0% → now in_progress
  65%. PDF + Markdown shipped (BrandCanvasPDFExport,
  MarkdownPDFExporter, BrandMarkdownExport,
  generate-brand-strategy-pdf). Word (.docx) is the remaining gap.
- F-003 Draft Canvas synthesis: was 45% → now 60%. Current code
  generates a unified doc; the Gen 3 Draft-vs-Forensic *tier*
  distinction is the remaining gap, not the synthesis itself.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/feature_status_tracker.xlsx
+++ b/docs/feature_status_tracker.xlsx
@@ -1071,7 +1071,7 @@
         </is>
       </c>
       <c r="H5" s="7" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>Edge function exists for canvas synthesis. DRAFT badge + Forensic upgrade CTA needs design pass.</t>
+          <t>generate-brand-strategy-document edge function ships a unified strategy doc today. The Gen 3 Draft-vs-Forensic *tier* split (lighter doc after Layer 1, heavier after Avatar Builder) is the gap — current code doesn't distinguish them yet. DRAFT badge + Forensic upgrade CTA still needs design.</t>
         </is>
       </c>
       <c r="O5" s="8" t="n">
@@ -1388,11 +1388,11 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>not_started</t>
+          <t>in_review</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
       <c r="J10" s="4" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>Differential vs Draft Canvas is the core demonstration of value.</t>
+          <t>Brand strategy doc generation is the Forensic Canvas synthesis in current code: generate-brand-strategy-document (1164 LoC, pgvector RAG, Haiku, client-side orchestration to avoid 150s timeout) + generate-brand-strategy-section + MarkdownExportService. Remaining: explicit 'Strategic Entry Point' Trigger Moment callout and the Draft↔Forensic toggle (F-008.4). Sub-feature percent should override this.</t>
         </is>
       </c>
       <c r="O10" s="8" t="n">
@@ -2335,11 +2335,11 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>not_started</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="I25" s="4" t="inlineStr"/>
       <c r="J25" s="4" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>Required to deliver the canvas-as-artifact promise.</t>
+          <t>PDF + Markdown shipped: BrandCanvasPDFExport, MarkdownPDFExporter, BrandMarkdownExport, generate-brand-strategy-pdf edge function. Word (.docx) export is the remaining gap. Once Draft/Forensic tier split lands in F-003/F-008, ensure both tiers export.</t>
         </is>
       </c>
       <c r="O25" s="8" t="n">

</xml_diff>

<commit_message>
feat(planning): add Problems sheet + problems_addressed column on Features
Adds a Problems sheet capturing the 10 grand-vision problems the app
solves for the user, each mapped to the features that help solve it.
fulfilment_status derives from mapped feature status (counts complete
and in_review against total). alpha_testable column flags which
problems Alpha-stage features can actually validate (P-001, P-002
Yes; P-003, P-005 Partial; rest No).

Problems sheet is the source of truth for the mapping; Features sheet
gets a derived problems_addressed column generated at build time so
the two sides can't drift.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/feature_status_tracker.xlsx
+++ b/docs/feature_status_tracker.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Features" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-features" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Phase Gate" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Brand Needs" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Risks" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Change Log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Problems" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Features" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sub-features" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Phase Gate" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Brand Needs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Risks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Change Log" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -158,14 +159,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFBDD7EE"/>
+          <fgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
+          <fgColor rgb="FFBDD7EE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -800,7 +801,560 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Problems — the grand-vision list, mapped to features</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Each problem is mapped to the features that help solve it. fulfilment_status derives from the status of mapped features. alpha_testable = whether Alpha-stage features alone are enough to validate this problem with testers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>problem_id</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>problem_statement</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>earliest_phase_solvable</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>alpha_testable</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>mapped_features</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>feature_count</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>complete_or_review_count</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>fulfilment_status</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>P-001</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Generic AI doesn't know my customer deeply enough.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Alpha</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>F-004,F-005,F-006,F-007,F-008,F-009,F-012,F-022</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="4">
+        <f>(COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-012",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-012",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review"))</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-012",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-012",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-012",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review"))=8,"MET",IF((COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-012",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-012",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review"))=0,"OPEN — 0 of 8","PARTIAL — "&amp;(COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-012",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-012",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review"))&amp;" of 8")))</f>
+        <v/>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Core Alpha thesis: Avatar Builder + Forensic Canvas produce a depth of customer understanding generic prompting can't reach. F-022 (Coach mode) extends this in Beta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>P-002</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>I don't know what to ask myself about my customer.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Alpha</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>F-001,F-004,F-005,F-006,F-007,F-009</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" s="4">
+        <f>(COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"in_review"))</f>
+        <v/>
+      </c>
+      <c r="H6" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"in_review"))=6,"MET",IF((COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"in_review"))=0,"OPEN — 0 of 6","PARTIAL — "&amp;(COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-001",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-004",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-005",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-009",'Features'!$G$3:$G$61,"in_review"))&amp;" of 6")))</f>
+        <v/>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>10-Q conversation + 4 Avatar Builder sections provide the inquiry structure. F-009 'Think About This' mode explicitly generates reflective questions per field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>P-003</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>My brand strategy doc is shallow or doesn't exist.</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Alpha</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>F-003,F-008,F-023,F-053</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="4">
+        <f>(COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review"))</f>
+        <v/>
+      </c>
+      <c r="H7" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review"))=4,"MET",IF((COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review"))=0,"OPEN — 0 of 4","PARTIAL — "&amp;(COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-003",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-023",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review"))&amp;" of 4")))</f>
+        <v/>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>F-008 (Forensic Canvas via generate-brand-strategy-document) is the primary fulfilment — substantially shipped. Polished Word export (F-023) and multi-angle (F-053) are Beta extensions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>P-004</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>My copy and creative aren't grounded in strategy.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>F-008,F-020,F-021,F-055</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" s="4">
+        <f>(COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))=4,"MET",IF((COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))=0,"OPEN — 0 of 4","PARTIAL — "&amp;(COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))&amp;" of 4")))</f>
+        <v/>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Requires Create mode outputs (F-020 Amazon, F-021 Voice Guide, F-055 Design brief). None ship in Alpha. The canvas (F-008) is the anchor but not the deliverable for this problem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>P-005</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>My customer's actual language doesn't make it into my copy.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>F-007,F-008,F-020,F-021</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="4">
+        <f>(COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"in_review"))</f>
+        <v/>
+      </c>
+      <c r="H9" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"in_review"))=4,"MET",IF((COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"in_review"))=0,"OPEN — 0 of 4","PARTIAL — "&amp;(COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-020",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-021",'Features'!$G$3:$G$61,"in_review"))&amp;" of 4")))</f>
+        <v/>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>F-007 Voice of Customer extracts verbatim language in Alpha. F-020/F-021 (Beta) consume it. Alpha can prove 'we capture the language'; only Beta proves 'it shows up in your copy'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>P-006</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>My existing image/video set is doing something — but I can't tell what's missing or off.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>F-006,F-007,F-054,F-055</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="4">
+        <f>(COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))</f>
+        <v/>
+      </c>
+      <c r="H10" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))=4,"MET",IF((COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))=0,"OPEN — 0 of 4","PARTIAL — "&amp;(COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-006",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-007",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))&amp;" of 4")))</f>
+        <v/>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>InfinityVault's specific need (N-002). F-054 is conditional on the asset-tracking decision gate. F-006/F-007 supply the 'what should this connect to' context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>P-007</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>I have no thinking partner who remembers my brand.</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>F-022,F-031,F-049</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="4">
+        <f>(COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-049",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-049",'Features'!$G$3:$G$61,"in_review"))</f>
+        <v/>
+      </c>
+      <c r="H11" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-049",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-049",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-049",'Features'!$G$3:$G$61,"in_review"))=3,"MET",IF((COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-049",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-049",'Features'!$G$3:$G$61,"in_review"))=0,"OPEN — 0 of 3","PARTIAL — "&amp;(COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-031",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-049",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-049",'Features'!$G$3:$G$61,"in_review"))&amp;" of 3")))</f>
+        <v/>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>F-022 Coach mode is the answer. RAG (F-049) makes the memory queryable. F-031 (My Brands) lets the partner know which brand we're discussing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>P-008</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>I can't cheaply test multiple positioning angles.</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>F-042,F-053,F-055</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="4">
+        <f>(COUNTIFS('Features'!$A$3:$A$61,"F-042",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-042",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))</f>
+        <v/>
+      </c>
+      <c r="H12" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-042",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-042",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-042",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))=3,"MET",IF((COUNTIFS('Features'!$A$3:$A$61,"F-042",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-042",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))=0,"OPEN — 0 of 3","PARTIAL — "&amp;(COUNTIFS('Features'!$A$3:$A$61,"F-042",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-042",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-055",'Features'!$G$3:$G$61,"in_review"))&amp;" of 3")))</f>
+        <v/>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>F-053 is the primary fulfilment. F-055 lets each angle drive its own design brief. F-042 comparison view (GA) lets the user A/B them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>P-009</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>I can't tell when my strategy and my live assets have drifted apart.</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>F-028,F-029,F-030,F-043,F-054</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" s="4">
+        <f>(COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-029",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-029",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-030",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-030",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-043",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-043",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"in_review"))</f>
+        <v/>
+      </c>
+      <c r="H13" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-029",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-030",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-043",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-029",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-029",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-030",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-030",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-043",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-043",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"in_review"))=5,"MET",IF((COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-029",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-029",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-030",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-030",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-043",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-043",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"in_review"))=0,"OPEN — 0 of 5","PARTIAL — "&amp;(COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-028",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-029",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-029",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-030",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-030",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-043",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-043",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-054",'Features'!$G$3:$G$61,"in_review"))&amp;" of 5")))</f>
+        <v/>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Conditional on the asset-tracking decision. F-043 field edit history adds the temporal dimension on the strategy side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>P-010</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Every marketing decision feels reactive.</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>F-008,F-022,F-038,F-053</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="4">
+        <f>(COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review"))</f>
+        <v/>
+      </c>
+      <c r="H14" s="4">
+        <f>IF((COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"blocked")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"blocked"))&gt;0,"BLOCKED — see mapped features",IF((COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review"))=4,"MET",IF((COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review"))=0,"OPEN — 0 of 4","PARTIAL — "&amp;(COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-008",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-022",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-038",'Features'!$G$3:$G$61,"in_review")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"complete")+COUNTIFS('Features'!$A$3:$A$61,"F-053",'Features'!$G$3:$G$61,"in_review"))&amp;" of 4")))</f>
+        <v/>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Forensic Canvas as North Star (F-008), Coach for ongoing decisions (F-022), performance metrics (F-038) close the loop. F-053 lets decisions live at the angle level.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="H5:H14">
+    <cfRule type="expression" priority="1" dxfId="2">
+      <formula>H5="MET"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>ISNUMBER(SEARCH("BLOCKED",H5))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>ISNUMBER(SEARCH("PARTIAL",H5))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>ISNUMBER(SEARCH("OPEN",H5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D5:D14">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="2">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="1">
+      <formula>"Partial"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="C5:C64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
+      <formula1>"Alpha,Beta,GA,Post-GA"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D5:D64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
+      <formula1>"Yes,Partial,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -814,10 +1368,11 @@
     <col width="32" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -885,20 +1440,25 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
+          <t>problems_addressed</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
           <t>effort_estimate_hours</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>actual_hours</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -954,18 +1514,23 @@
           <t>F-018</t>
         </is>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>P-002</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="M3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>Existing chat infrastructure (SupabaseChatService) is the substrate. Needs Trevor-voice prompt set + 10-Q question script wired.</t>
         </is>
       </c>
-      <c r="O3" s="8" t="n">
+      <c r="P3" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1019,18 +1584,19 @@
           <t>F-001,F-012</t>
         </is>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Field extraction pipeline exists; sidebar render needs to subscribe to extraction events.</t>
         </is>
       </c>
-      <c r="O4" s="8" t="n">
+      <c r="P4" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1084,18 +1650,23 @@
           <t>F-001,F-018</t>
         </is>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>P-003</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>generate-brand-strategy-document edge function ships a unified strategy doc today. The Gen 3 Draft-vs-Forensic *tier* split (lighter doc after Layer 1, heavier after Avatar Builder) is the gap — current code doesn't distinguish them yet. DRAFT badge + Forensic upgrade CTA still needs design.</t>
         </is>
       </c>
-      <c r="O5" s="8" t="n">
+      <c r="P5" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1149,18 +1720,23 @@
           <t>F-003,F-009</t>
         </is>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>P-001,P-002</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>Gen 3 spec is the source of truth. Existing V2 PRD predates Gen 3; verify field list.</t>
         </is>
       </c>
-      <c r="O6" s="8" t="n">
+      <c r="P6" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1214,14 +1790,19 @@
           <t>F-004</t>
         </is>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>P-001,P-002</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="M7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="4" t="inlineStr"/>
-      <c r="O7" s="8" t="n">
+      <c r="N7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="4" t="inlineStr"/>
+      <c r="P7" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1275,18 +1856,23 @@
           <t>F-005</t>
         </is>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>P-001,P-002,P-006</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="N8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>Trigger Moment is Trevor's flagged most-important field — must surface prominently.</t>
         </is>
       </c>
-      <c r="O8" s="8" t="n">
+      <c r="P8" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1340,18 +1926,23 @@
           <t>F-006</t>
         </is>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>P-001,P-002,P-005,P-006</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="M9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>Requires voice-of-customer-analysis edge function.</t>
         </is>
       </c>
-      <c r="O9" s="8" t="n">
+      <c r="P9" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1405,18 +1996,23 @@
           <t>F-004,F-005,F-006,F-007</t>
         </is>
       </c>
-      <c r="L10" s="4" t="n">
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>P-001,P-003,P-004,P-005,P-010</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="M10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="N10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>Brand strategy doc generation is the Forensic Canvas synthesis in current code: generate-brand-strategy-document (1164 LoC, pgvector RAG, Haiku, client-side orchestration to avoid 150s timeout) + generate-brand-strategy-section + MarkdownExportService. Remaining: explicit 'Strategic Entry Point' Trigger Moment callout and the Draft↔Forensic toggle (F-008.4). Sub-feature percent should override this.</t>
         </is>
       </c>
-      <c r="O10" s="8" t="n">
+      <c r="P10" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1470,18 +2066,23 @@
           <t>F-018</t>
         </is>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>P-001,P-002</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="M11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="N11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
         <is>
           <t>AIAssistant component exists for V2 fields; needs Gen 3 mode expansion.</t>
         </is>
       </c>
-      <c r="O11" s="8" t="n">
+      <c r="P11" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1531,18 +2132,19 @@
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr"/>
-      <c r="L12" s="4" t="n">
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="N12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>Existing V2 UI is form-shaped. Trevor's Risk Register flag: 'feels like a form, not a conversation' is Critical.</t>
         </is>
       </c>
-      <c r="O12" s="8" t="n">
+      <c r="P12" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1592,18 +2194,19 @@
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr"/>
-      <c r="L13" s="4" t="n">
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="N13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>Trust foundation per Trevor + existing PRD constraint. Partially present in V2 quality badge code.</t>
         </is>
       </c>
-      <c r="O13" s="8" t="n">
+      <c r="P13" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1653,18 +2256,23 @@
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr"/>
-      <c r="L14" s="4" t="n">
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>P-001</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="M14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="N14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>Field extraction shipped recently (commit 77ae116 — IDEA Brand Coach quality score badges).</t>
         </is>
       </c>
-      <c r="O14" s="8" t="n">
+      <c r="P14" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1718,18 +2326,19 @@
           <t>F-003,F-017</t>
         </is>
       </c>
-      <c r="L15" s="4" t="n">
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="N15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
         <is>
           <t>Spec lives in Launch Roadmap › Feedback Loop sheet.</t>
         </is>
       </c>
-      <c r="O15" s="8" t="n">
+      <c r="P15" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1783,18 +2392,19 @@
           <t>F-008,F-017</t>
         </is>
       </c>
-      <c r="L16" s="4" t="n">
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="N16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>% selecting 'update existing assets' is the Alpha→Beta asset-tracking gate.</t>
         </is>
       </c>
-      <c r="O16" s="8" t="n">
+      <c r="P16" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1848,18 +2458,19 @@
           <t>F-017</t>
         </is>
       </c>
-      <c r="L17" s="4" t="n">
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="4" t="inlineStr">
+      <c r="N17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
         <is>
           <t>Requires scheduled-send infrastructure (Resend / Supabase cron).</t>
         </is>
       </c>
-      <c r="O17" s="8" t="n">
+      <c r="P17" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1909,18 +2520,19 @@
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="n">
+      <c r="L18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="N18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>Single destination simplifies the alpha findings synthesis step.</t>
         </is>
       </c>
-      <c r="O18" s="8" t="n">
+      <c r="P18" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -1970,18 +2582,19 @@
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr"/>
-      <c r="L19" s="4" t="n">
+      <c r="L19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="M19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="N19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
         <is>
           <t>Cheap to install. Risk Register flags that testers won't report half the bugs.</t>
         </is>
       </c>
-      <c r="O19" s="8" t="n">
+      <c r="P19" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2031,18 +2644,19 @@
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr"/>
-      <c r="L20" s="4" t="n">
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="N20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>No tutorial. Sets expectation that this is alpha and feedback is the deliverable.</t>
         </is>
       </c>
-      <c r="O20" s="8" t="n">
+      <c r="P20" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2096,18 +2710,19 @@
           <t>F-008</t>
         </is>
       </c>
-      <c r="L21" s="4" t="n">
+      <c r="L21" s="4" t="inlineStr"/>
+      <c r="M21" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="M21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="N21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>Central conversion test of beta. Pay-gate previews must use real canvas data.</t>
         </is>
       </c>
-      <c r="O21" s="8" t="n">
+      <c r="P21" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2161,18 +2776,23 @@
           <t>F-008,F-019</t>
         </is>
       </c>
-      <c r="L22" s="4" t="n">
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>P-004,P-005</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="M22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="N22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>First Create-mode output. Anchors the pay-gate preview.</t>
         </is>
       </c>
-      <c r="O22" s="8" t="n">
+      <c r="P22" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2226,14 +2846,19 @@
           <t>F-008,F-019</t>
         </is>
       </c>
-      <c r="L23" s="4" t="n">
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>P-004,P-005</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M23" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="4" t="inlineStr"/>
-      <c r="O23" s="8" t="n">
+      <c r="N23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="4" t="inlineStr"/>
+      <c r="P23" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2287,18 +2912,23 @@
           <t>F-008</t>
         </is>
       </c>
-      <c r="L24" s="4" t="n">
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>P-001,P-007,P-010</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="M24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="N24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>Required to deliver the £29/mo subscription value prop per Trevor's spec.</t>
         </is>
       </c>
-      <c r="O24" s="8" t="n">
+      <c r="P24" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2352,18 +2982,23 @@
           <t>F-003,F-008</t>
         </is>
       </c>
-      <c r="L25" s="4" t="n">
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>P-003</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M25" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="4" t="inlineStr">
+      <c r="N25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
         <is>
           <t>PDF + Markdown shipped: BrandCanvasPDFExport, MarkdownPDFExporter, BrandMarkdownExport, generate-brand-strategy-pdf edge function. Word (.docx) export is the remaining gap. Once Draft/Forensic tier split lands in F-003/F-008, ensure both tiers export.</t>
         </is>
       </c>
-      <c r="O25" s="8" t="n">
+      <c r="P25" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2413,18 +3048,19 @@
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr"/>
-      <c r="L26" s="4" t="n">
+      <c r="L26" s="4" t="inlineStr"/>
+      <c r="M26" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="M26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="N26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
         <is>
           <t>Conversion data is the whole point of beta.</t>
         </is>
       </c>
-      <c r="O26" s="8" t="n">
+      <c r="P26" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2474,18 +3110,19 @@
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr"/>
-      <c r="L27" s="4" t="n">
+      <c r="L27" s="4" t="inlineStr"/>
+      <c r="M27" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="4" t="inlineStr">
+      <c r="N27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>Refund-rate risk is partly a support-responsiveness problem.</t>
         </is>
       </c>
-      <c r="O27" s="8" t="n">
+      <c r="P27" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2539,18 +3176,19 @@
           <t>F-015</t>
         </is>
       </c>
-      <c r="L28" s="4" t="n">
+      <c r="L28" s="4" t="inlineStr"/>
+      <c r="M28" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="4" t="inlineStr">
+      <c r="N28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="4" t="inlineStr">
         <is>
           <t>Target: 5+ verified testimonials by end of Beta; 10+ within 3 months.</t>
         </is>
       </c>
-      <c r="O28" s="8" t="n">
+      <c r="P28" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2600,18 +3238,19 @@
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr"/>
-      <c r="L29" s="4" t="n">
+      <c r="L29" s="4" t="inlineStr"/>
+      <c r="M29" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="M29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="4" t="inlineStr">
+      <c r="N29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
         <is>
           <t>Diagnostic largely exists (FreeDiagnostic + BetaFeedback components). Handoff into Layer 1 still loose.</t>
         </is>
       </c>
-      <c r="O29" s="8" t="n">
+      <c r="P29" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2669,18 +3308,23 @@
           <t>F-014</t>
         </is>
       </c>
-      <c r="L30" s="4" t="n">
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>P-009</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="M30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="4" t="inlineStr">
+      <c r="N30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
         <is>
           <t>DEFERRED DECISION. Gate at end of Alpha. Default is NO. Trevor's Gen 3 spec does not include asset tracking — only ship if Moment 2 signal is ≥40%.</t>
         </is>
       </c>
-      <c r="O30" s="8" t="n">
+      <c r="P30" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2738,18 +3382,23 @@
           <t>F-028</t>
         </is>
       </c>
-      <c r="L31" s="4" t="n">
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>P-009</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="M31" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
+      <c r="N31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
         <is>
           <t>Introduces the temporal signal — user can see what's out of date.</t>
         </is>
       </c>
-      <c r="O31" s="8" t="n">
+      <c r="P31" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2807,18 +3456,23 @@
           <t>F-029</t>
         </is>
       </c>
-      <c r="L32" s="4" t="n">
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>P-009</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="M32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" s="4" t="inlineStr">
+      <c r="N32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
         <is>
           <t>Likely a GA-era feature per brief; listed for completeness.</t>
         </is>
       </c>
-      <c r="O32" s="8" t="n">
+      <c r="P32" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2872,18 +3526,23 @@
           <t>F-046</t>
         </is>
       </c>
-      <c r="L33" s="4" t="n">
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>P-007</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="M33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" s="4" t="inlineStr">
+      <c r="N33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
         <is>
           <t>Power users will have multiple brands; product caps out at one customer without this.</t>
         </is>
       </c>
-      <c r="O33" s="8" t="n">
+      <c r="P33" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2937,18 +3596,19 @@
           <t>F-027</t>
         </is>
       </c>
-      <c r="L34" s="4" t="n">
+      <c r="L34" s="4" t="inlineStr"/>
+      <c r="M34" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="M34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" s="4" t="inlineStr">
+      <c r="N34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
         <is>
           <t>Top-of-funnel users drop off without this.</t>
         </is>
       </c>
-      <c r="O34" s="8" t="n">
+      <c r="P34" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -2998,18 +3658,19 @@
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr"/>
-      <c r="L35" s="4" t="n">
+      <c r="L35" s="4" t="inlineStr"/>
+      <c r="M35" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="M35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="4" t="inlineStr">
+      <c r="N35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
         <is>
           <t>Public launch means support cost scales with users — self-serve protects margin.</t>
         </is>
       </c>
-      <c r="O35" s="8" t="n">
+      <c r="P35" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3063,18 +3724,19 @@
           <t>F-019</t>
         </is>
       </c>
-      <c r="L36" s="4" t="n">
+      <c r="L36" s="4" t="inlineStr"/>
+      <c r="M36" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="M36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" s="4" t="inlineStr">
+      <c r="N36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
         <is>
           <t>Conversion surface for non-warm visitors.</t>
         </is>
       </c>
-      <c r="O36" s="8" t="n">
+      <c r="P36" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3124,18 +3786,19 @@
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr"/>
-      <c r="L37" s="4" t="n">
+      <c r="L37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M37" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" s="4" t="inlineStr">
+      <c r="N37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
         <is>
           <t>Trust signal required for paid users.</t>
         </is>
       </c>
-      <c r="O37" s="8" t="n">
+      <c r="P37" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3189,18 +3852,19 @@
           <t>F-025</t>
         </is>
       </c>
-      <c r="L38" s="4" t="n">
+      <c r="L38" s="4" t="inlineStr"/>
+      <c r="M38" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" s="4" t="inlineStr">
+      <c r="N38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
         <is>
           <t>Reduces ticket volume and improves time-to-value.</t>
         </is>
       </c>
-      <c r="O38" s="8" t="n">
+      <c r="P38" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3250,18 +3914,19 @@
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr"/>
-      <c r="L39" s="4" t="n">
+      <c r="L39" s="4" t="inlineStr"/>
+      <c r="M39" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M39" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" s="4" t="inlineStr">
+      <c r="N39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
         <is>
           <t>Legal hygiene required for paid public product.</t>
         </is>
       </c>
-      <c r="O39" s="8" t="n">
+      <c r="P39" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3315,18 +3980,23 @@
           <t>F-046</t>
         </is>
       </c>
-      <c r="L40" s="4" t="n">
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>P-010</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="M40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N40" s="4" t="inlineStr">
+      <c r="N40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
         <is>
           <t>OPEN QUESTION: existing V2 PRD scopes this as a P0 V2 feature. Trevor's Gen 3 spec does not address it. Treated here as GA P0; needs Matthew sign-off.</t>
         </is>
       </c>
-      <c r="O40" s="8" t="n">
+      <c r="P40" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3380,18 +4050,19 @@
           <t>F-019</t>
         </is>
       </c>
-      <c r="L41" s="4" t="n">
+      <c r="L41" s="4" t="inlineStr"/>
+      <c r="M41" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M41" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N41" s="4" t="inlineStr">
+      <c r="N41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
         <is>
           <t>Acquisition lever from GA Plan.</t>
         </is>
       </c>
-      <c r="O41" s="8" t="n">
+      <c r="P41" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3441,18 +4112,19 @@
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="4" t="n">
+      <c r="L42" s="4" t="inlineStr"/>
+      <c r="M42" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M42" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N42" s="4" t="inlineStr">
+      <c r="N42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
         <is>
           <t>Brand strategist partner channel needs attribution before outreach.</t>
         </is>
       </c>
-      <c r="O42" s="8" t="n">
+      <c r="P42" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3502,18 +4174,19 @@
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr"/>
-      <c r="L43" s="4" t="n">
+      <c r="L43" s="4" t="inlineStr"/>
+      <c r="M43" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="M43" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N43" s="4" t="inlineStr">
+      <c r="N43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
         <is>
           <t>Three-month organic ramp — start at beginning of beta to earn GA traffic.</t>
         </is>
       </c>
-      <c r="O43" s="8" t="n">
+      <c r="P43" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3567,18 +4240,23 @@
           <t>F-031</t>
         </is>
       </c>
-      <c r="L44" s="4" t="n">
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>P-008</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M44" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N44" s="4" t="inlineStr">
+      <c r="N44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
         <is>
           <t>Power-user feature; rewards multi-canvas usage.</t>
         </is>
       </c>
-      <c r="O44" s="8" t="n">
+      <c r="P44" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3632,18 +4310,23 @@
           <t>F-046</t>
         </is>
       </c>
-      <c r="L45" s="4" t="n">
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>P-009</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="M45" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N45" s="4" t="inlineStr">
+      <c r="N45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
         <is>
           <t>Schema needs field_edit_history table.</t>
         </is>
       </c>
-      <c r="O45" s="8" t="n">
+      <c r="P45" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3697,18 +4380,19 @@
           <t>F-031</t>
         </is>
       </c>
-      <c r="L46" s="4" t="n">
+      <c r="L46" s="4" t="inlineStr"/>
+      <c r="M46" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="M46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N46" s="4" t="inlineStr">
+      <c r="N46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
         <is>
           <t>Power-user feature.</t>
         </is>
       </c>
-      <c r="O46" s="8" t="n">
+      <c r="P46" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3762,18 +4446,19 @@
           <t>F-034</t>
         </is>
       </c>
-      <c r="L47" s="4" t="n">
+      <c r="L47" s="4" t="inlineStr"/>
+      <c r="M47" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N47" s="4" t="inlineStr">
+      <c r="N47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
         <is>
           <t>TikTok integration is GA+4wks per Launch Roadmap; not a build dependency.</t>
         </is>
       </c>
-      <c r="O47" s="8" t="n">
+      <c r="P47" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3827,14 +4512,15 @@
           <t>F-024</t>
         </is>
       </c>
-      <c r="L48" s="4" t="n">
+      <c r="L48" s="4" t="inlineStr"/>
+      <c r="M48" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M48" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N48" s="4" t="inlineStr"/>
-      <c r="O48" s="8" t="n">
+      <c r="N48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" s="4" t="inlineStr"/>
+      <c r="P48" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3884,14 +4570,15 @@
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr"/>
-      <c r="L49" s="4" t="n">
+      <c r="L49" s="4" t="inlineStr"/>
+      <c r="M49" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M49" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N49" s="4" t="inlineStr"/>
-      <c r="O49" s="8" t="n">
+      <c r="N49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" s="4" t="inlineStr"/>
+      <c r="P49" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3941,18 +4628,19 @@
         </is>
       </c>
       <c r="K50" s="4" t="inlineStr"/>
-      <c r="L50" s="4" t="n">
+      <c r="L50" s="4" t="inlineStr"/>
+      <c r="M50" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M50" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N50" s="4" t="inlineStr">
+      <c r="N50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="4" t="inlineStr">
         <is>
           <t>Pairs with UTM data to triangulate true attribution.</t>
         </is>
       </c>
-      <c r="O50" s="8" t="n">
+      <c r="P50" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4002,18 +4690,19 @@
         </is>
       </c>
       <c r="K51" s="4" t="inlineStr"/>
-      <c r="L51" s="4" t="n">
+      <c r="L51" s="4" t="inlineStr"/>
+      <c r="M51" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M51" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N51" s="4" t="inlineStr">
+      <c r="N51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" s="4" t="inlineStr">
         <is>
           <t>Additive only. RLS policies in F-047.</t>
         </is>
       </c>
-      <c r="O51" s="8" t="n">
+      <c r="P51" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4067,14 +4756,15 @@
           <t>F-046</t>
         </is>
       </c>
-      <c r="L52" s="4" t="n">
+      <c r="L52" s="4" t="inlineStr"/>
+      <c r="M52" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M52" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N52" s="4" t="inlineStr"/>
-      <c r="O52" s="8" t="n">
+      <c r="N52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" s="4" t="inlineStr"/>
+      <c r="P52" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4124,18 +4814,19 @@
         </is>
       </c>
       <c r="K53" s="4" t="inlineStr"/>
-      <c r="L53" s="4" t="n">
+      <c r="L53" s="4" t="inlineStr"/>
+      <c r="M53" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="M53" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N53" s="4" t="inlineStr">
+      <c r="N53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" s="4" t="inlineStr">
         <is>
           <t>idea-framework-consultant exists; Gen 3 functions partially overlap. Audit needed.</t>
         </is>
       </c>
-      <c r="O53" s="8" t="n">
+      <c r="P53" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4189,18 +4880,23 @@
           <t>F-048</t>
         </is>
       </c>
-      <c r="L54" s="4" t="n">
+      <c r="L54" s="4" t="inlineStr">
+        <is>
+          <t>P-007</t>
+        </is>
+      </c>
+      <c r="M54" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="M54" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" s="4" t="inlineStr">
+      <c r="N54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="4" t="inlineStr">
         <is>
           <t>OpenAI embeddings removed in commit 260128b (consolidated to Claude/internal embeddings) — verify RAG pipeline still wired.</t>
         </is>
       </c>
-      <c r="O54" s="8" t="n">
+      <c r="P54" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4250,18 +4946,19 @@
         </is>
       </c>
       <c r="K55" s="4" t="inlineStr"/>
-      <c r="L55" s="4" t="n">
+      <c r="L55" s="4" t="inlineStr"/>
+      <c r="M55" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M55" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" s="4" t="inlineStr">
+      <c r="N55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="4" t="inlineStr">
         <is>
           <t>Hook already exists. Audit V2 routes for missing gates.</t>
         </is>
       </c>
-      <c r="O55" s="8" t="n">
+      <c r="P55" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4311,18 +5008,19 @@
         </is>
       </c>
       <c r="K56" s="4" t="inlineStr"/>
-      <c r="L56" s="4" t="n">
+      <c r="L56" s="4" t="inlineStr"/>
+      <c r="M56" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="M56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N56" s="4" t="inlineStr">
+      <c r="N56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="4" t="inlineStr">
         <is>
           <t>Refactor patterns shipped (SupabaseChatService split, FieldSyncService, AIAssistant decomposition). Verify all Gen 3 work picks up new patterns.</t>
         </is>
       </c>
-      <c r="O56" s="8" t="n">
+      <c r="P56" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4376,18 +5074,23 @@
           <t>F-008,F-031</t>
         </is>
       </c>
-      <c r="L57" s="4" t="n">
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>P-003,P-008,P-010</t>
+        </is>
+      </c>
+      <c r="M57" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="M57" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N57" s="4" t="inlineStr">
+      <c r="N57" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" s="4" t="inlineStr">
         <is>
           <t>Validates A/B angle testing for paying users. Each angle = a strategy variant tied to a canonical avatar. Surfaces in Coach mode and Export. OPEN: schema choice — separate canvases per angle vs angle-tagged sections within one canvas.</t>
         </is>
       </c>
-      <c r="O57" s="8" t="n">
+      <c r="P57" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4445,18 +5148,23 @@
           <t>F-028,F-053</t>
         </is>
       </c>
-      <c r="L58" s="4" t="n">
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>P-006,P-009</t>
+        </is>
+      </c>
+      <c r="M58" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="M58" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N58" s="4" t="inlineStr">
+      <c r="N58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" s="4" t="inlineStr">
         <is>
           <t>Extension of asset_tracking that goes beyond text. Anchored to InfinityVault need N-002 (assess images/videos, identify what's missing, surface emotional-connection opportunities). Requires image storage (Supabase Storage) and a comparison UI.</t>
         </is>
       </c>
-      <c r="O58" s="8" t="n">
+      <c r="P58" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4510,18 +5218,23 @@
           <t>F-008,F-053</t>
         </is>
       </c>
-      <c r="L59" s="4" t="n">
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>P-004,P-006,P-008</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="M59" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N59" s="4" t="inlineStr">
+      <c r="N59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" s="4" t="inlineStr">
         <is>
           <t>Sibling to F-020 (Amazon listing copy) and F-021 (Brand Voice Guide). Bridges the canvas to creative work. Required to make F-054 actionable (gap → brief → asset).</t>
         </is>
       </c>
-      <c r="O59" s="8" t="n">
+      <c r="P59" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4575,18 +5288,19 @@
           <t>F-055</t>
         </is>
       </c>
-      <c r="L60" s="4" t="n">
+      <c r="L60" s="4" t="inlineStr"/>
+      <c r="M60" s="4" t="n">
         <v>80</v>
       </c>
-      <c r="M60" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N60" s="4" t="inlineStr">
+      <c r="N60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" s="4" t="inlineStr">
         <is>
           <t>Surfaced as 'coming soon' in UI (teaser). Closes the loop from canvas → design brief → generated imagery. No model choice locked in; defer until Post-GA stability work is done.</t>
         </is>
       </c>
-      <c r="O60" s="8" t="n">
+      <c r="P60" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -4640,30 +5354,31 @@
         </is>
       </c>
       <c r="K61" s="4" t="inlineStr"/>
-      <c r="L61" s="4" t="n">
+      <c r="L61" s="4" t="inlineStr"/>
+      <c r="M61" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M61" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N61" s="4" t="inlineStr">
+      <c r="N61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" s="4" t="inlineStr">
         <is>
           <t>DEFERRED DECISION. Trevor's Gen 3 Brief specifies Lovable; existing codebase is React + Supabase. Don't half-port. Default: extend existing repo until Matthew decides otherwise.</t>
         </is>
       </c>
-      <c r="O61" s="8" t="n">
+      <c r="P61" s="8" t="n">
         <v>46155</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:P1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:G261">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"complete"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
       <formula>"in_review"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
@@ -4672,7 +5387,7 @@
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
       <formula>"blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
       <formula>"not_started"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4694,7 +5409,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7624,7 +8339,7 @@
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"complete"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
       <formula>"in_review"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
@@ -7633,7 +8348,7 @@
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
       <formula>"blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
       <formula>"not_started"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7646,7 +8361,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8515,7 +9230,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8722,7 +9437,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9415,7 +10130,7 @@
     <mergeCell ref="A1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="E4:E117">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"monitoring"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
@@ -9438,7 +10153,7 @@
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="1">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="3">
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9457,13 +10172,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9545,6 +10260,28 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Matthew (via Claude Code)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Corrected status for brand strategy doc + PDF export; added Problems sheet</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>F-008 was wrongly marked not_started — corrected to in_review 80% based on shipped generate-brand-strategy-document. F-023 corrected to in_progress 65% (PDF + Markdown shipped, Word still missing). Added Problems sheet with the 10 problems we solve mapped to features; added problems_addressed column on Features.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
chore(planning): set workbook TODAY to 2026-05-16
Updates last_updated on all feature rows and corrects the latest
Change Log entry's date.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/feature_status_tracker.xlsx
+++ b/docs/feature_status_tracker.xlsx
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="P3" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="P4" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="P5" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="P6" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr"/>
       <c r="P7" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="P8" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="P9" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="P10" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
@@ -2083,7 +2083,7 @@
         </is>
       </c>
       <c r="P11" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="P12" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="P13" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
@@ -2273,7 +2273,7 @@
         </is>
       </c>
       <c r="P14" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1">
@@ -2339,7 +2339,7 @@
         </is>
       </c>
       <c r="P15" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1">
@@ -2405,7 +2405,7 @@
         </is>
       </c>
       <c r="P16" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1">
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="P17" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="P18" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
@@ -2595,7 +2595,7 @@
         </is>
       </c>
       <c r="P19" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1">
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="P20" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1">
@@ -2723,7 +2723,7 @@
         </is>
       </c>
       <c r="P21" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1">
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="P22" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr"/>
       <c r="P23" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="P24" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1">
@@ -2999,7 +2999,7 @@
         </is>
       </c>
       <c r="P25" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="26" ht="42" customHeight="1">
@@ -3061,7 +3061,7 @@
         </is>
       </c>
       <c r="P26" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="27" ht="42" customHeight="1">
@@ -3123,7 +3123,7 @@
         </is>
       </c>
       <c r="P27" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="28" ht="42" customHeight="1">
@@ -3189,7 +3189,7 @@
         </is>
       </c>
       <c r="P28" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="29" ht="42" customHeight="1">
@@ -3251,7 +3251,7 @@
         </is>
       </c>
       <c r="P29" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="30" ht="42" customHeight="1">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="P30" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="31" ht="42" customHeight="1">
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="P31" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="32" ht="42" customHeight="1">
@@ -3473,7 +3473,7 @@
         </is>
       </c>
       <c r="P32" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="33" ht="42" customHeight="1">
@@ -3543,7 +3543,7 @@
         </is>
       </c>
       <c r="P33" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="34" ht="42" customHeight="1">
@@ -3609,7 +3609,7 @@
         </is>
       </c>
       <c r="P34" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="35" ht="42" customHeight="1">
@@ -3671,7 +3671,7 @@
         </is>
       </c>
       <c r="P35" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="36" ht="42" customHeight="1">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="P36" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="37" ht="42" customHeight="1">
@@ -3799,7 +3799,7 @@
         </is>
       </c>
       <c r="P37" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="38" ht="42" customHeight="1">
@@ -3865,7 +3865,7 @@
         </is>
       </c>
       <c r="P38" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="39" ht="42" customHeight="1">
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="P39" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="40" ht="42" customHeight="1">
@@ -3997,7 +3997,7 @@
         </is>
       </c>
       <c r="P40" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="41" ht="42" customHeight="1">
@@ -4063,7 +4063,7 @@
         </is>
       </c>
       <c r="P41" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="42" ht="42" customHeight="1">
@@ -4125,7 +4125,7 @@
         </is>
       </c>
       <c r="P42" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="43" ht="42" customHeight="1">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="P43" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="44" ht="42" customHeight="1">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="P44" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="45" ht="42" customHeight="1">
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="P45" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="46" ht="42" customHeight="1">
@@ -4393,7 +4393,7 @@
         </is>
       </c>
       <c r="P46" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="47" ht="42" customHeight="1">
@@ -4459,7 +4459,7 @@
         </is>
       </c>
       <c r="P47" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="48" ht="42" customHeight="1">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="O48" s="4" t="inlineStr"/>
       <c r="P48" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="49" ht="42" customHeight="1">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="O49" s="4" t="inlineStr"/>
       <c r="P49" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="50" ht="42" customHeight="1">
@@ -4641,7 +4641,7 @@
         </is>
       </c>
       <c r="P50" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="51" ht="42" customHeight="1">
@@ -4703,7 +4703,7 @@
         </is>
       </c>
       <c r="P51" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="52" ht="42" customHeight="1">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="O52" s="4" t="inlineStr"/>
       <c r="P52" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="53" ht="42" customHeight="1">
@@ -4827,7 +4827,7 @@
         </is>
       </c>
       <c r="P53" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="54" ht="42" customHeight="1">
@@ -4897,7 +4897,7 @@
         </is>
       </c>
       <c r="P54" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="55" ht="42" customHeight="1">
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="P55" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="56" ht="42" customHeight="1">
@@ -5021,7 +5021,7 @@
         </is>
       </c>
       <c r="P56" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="57" ht="42" customHeight="1">
@@ -5091,7 +5091,7 @@
         </is>
       </c>
       <c r="P57" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="58" ht="42" customHeight="1">
@@ -5165,7 +5165,7 @@
         </is>
       </c>
       <c r="P58" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="59" ht="42" customHeight="1">
@@ -5235,7 +5235,7 @@
         </is>
       </c>
       <c r="P59" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="60" ht="42" customHeight="1">
@@ -5301,7 +5301,7 @@
         </is>
       </c>
       <c r="P60" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="61" ht="42" customHeight="1">
@@ -5367,7 +5367,7 @@
         </is>
       </c>
       <c r="P61" s="8" t="n">
-        <v>46155</v>
+        <v>46158</v>
       </c>
     </row>
   </sheetData>
@@ -10263,7 +10263,7 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat(planning): add R-015 'product doesn't solve enough user problems' risk
Meta-risk above R-003 (form not conversation) and R-007 (no
testimonials). Severity Critical, exposed across all phases.

Trigger thresholds tied directly to the Problems sheet:
- <2 of {P-001, P-002, P-003} PARTIAL+ at Alpha exit
- <50% of testers articulate a concrete change in how they think
  about their customer
- <60% of shipped features map to ≥1 problem

Mitigation references the Problems sheet as the operational tool.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/feature_status_tracker.xlsx
+++ b/docs/feature_status_tracker.xlsx
@@ -9443,7 +9443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10125,11 +10125,58 @@
       </c>
       <c r="I17" s="4" t="inlineStr"/>
     </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>R-015</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Product doesn't solve enough user problems well enough to earn value</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>At Alpha exit, fewer than 2 of {P-001, P-002, P-003} verified PARTIAL+ via tester debriefs; OR &lt;50% of testers can articulate one concrete way the canvas changed how they think about their customer; OR fewer than 60% of shipped features map to ≥1 problem.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Matthew</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Problems sheet operationalises tracking. Alpha feedback Moments 1 + 2 measure perceived value directly. If signal is low at Alpha midpoint, narrow scope to deepen 1-2 problems rather than adding features.</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Meta-risk above R-003 (form not conversation) and R-007 (no testimonials). The failure mode where every feature ships on time but the product still doesn't matter to anyone. Operational tool: the Problems sheet — every feature should tag to at least one problem.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:E117">
+  <conditionalFormatting sqref="E4:E118">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"monitoring"</formula>
     </cfRule>
@@ -10143,7 +10190,7 @@
       <formula>"resolved"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4:D117">
+  <conditionalFormatting sqref="D4:D118">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="5">
       <formula>"Critical"</formula>
     </cfRule>
@@ -10158,13 +10205,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="C4:C117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
+    <dataValidation sqref="C4:C118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
       <formula1>"Alpha,Beta,GA,Post-GA,All"</formula1>
     </dataValidation>
-    <dataValidation sqref="D4:D117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
+    <dataValidation sqref="D4:D118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
+    <dataValidation sqref="E4:E118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must match one of the allowed options." type="list">
       <formula1>"monitoring,triggered,mitigated,resolved"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
refactor(planning): promote meta-risk to R-001; renumber Risks
Promotes 'Product doesn't solve enough user problems well enough to
earn value' to R-001 — it's the meta-risk that R-004 (form not
conversation) and R-008 (no testimonials) are specific symptoms of.

All 14 existing risks shift down by one. Cross-references inside risk
notes updated (R-001's note now references R-004 and R-008 by their
new ids; R-004 and R-008 notes mark themselves as symptoms of R-001).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/feature_status_tracker.xlsx
+++ b/docs/feature_status_tracker.xlsx
@@ -9519,17 +9519,17 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Alpha testers don't complete the flow</t>
+          <t>Product doesn't solve enough user problems well enough to earn value</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Alpha</t>
+          <t>All</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -9539,7 +9539,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>&lt;5 of 8 complete full flow by day 7</t>
+          <t>At Alpha exit, fewer than 2 of {P-001, P-002, P-003} verified PARTIAL+ via tester debriefs; OR &lt;50% of testers can articulate one concrete way the canvas changed how they think about their customer; OR fewer than 60% of shipped features map to ≥1 problem.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -9549,10 +9549,14 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Pre-flight QA checklist + daily monitoring + aggressive debrief follow-up planned</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr"/>
+          <t>Problems sheet operationalises tracking. Alpha feedback Moments 1 + 2 measure perceived value directly. If signal is low at Alpha midpoint, narrow scope to deepen 1-2 problems rather than adding features.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Meta-risk above R-004 (form not conversation) and R-008 (no testimonials). The failure mode where every feature ships on time but the product still doesn't matter to anyone. Operational tool: the Problems sheet — every feature should tag to at least one problem.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -9562,7 +9566,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Trevor's voice doesn't land for younger demographic</t>
+          <t>Alpha testers don't complete the flow</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -9572,7 +9576,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -9582,17 +9586,17 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>3+ testers flag 'sounds old' or 'corporate'</t>
+          <t>&lt;5 of 8 complete full flow by day 7</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Trevor</t>
+          <t>Matthew</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Mixed-experience tester pool; tone question in feedback Moment 1</t>
+          <t>Pre-flight QA checklist + daily monitoring + aggressive debrief follow-up planned</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr"/>
@@ -9605,7 +9609,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Avatar Builder feels like a form not a conversation</t>
+          <t>Trevor's voice doesn't land for younger demographic</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -9615,7 +9619,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -9625,24 +9629,20 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Any tester says 'this is just a long form'</t>
+          <t>3+ testers flag 'sounds old' or 'corporate'</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Matthew</t>
+          <t>Trevor</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>F-009 AI assistance wired before alpha; F-010 progressive disclosure tested; question phrasing reviewed by Trevor</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Kills Trevor's core thesis if it materialises.</t>
-        </is>
-      </c>
+          <t>Mixed-experience tester pool; tone question in feedback Moment 1</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr"/>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -9652,12 +9652,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Pay gate conversion too low</t>
+          <t>Avatar Builder feels like a form not a conversation</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Beta</t>
+          <t>Alpha</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>&lt;8% Draft viewers convert at 4-week mark</t>
+          <t>Any tester says 'this is just a long form'</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -9682,10 +9682,14 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Pay-gate previews use actual canvas data; pricing differentiated by job not features; A/B test framing</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr"/>
+          <t>F-009 AI assistance wired before alpha; F-010 progressive disclosure tested; question phrasing reviewed by Trevor</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Kills Trevor's core thesis if it materialises. Specific symptom of R-001.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -9695,7 +9699,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Refund rate is high</t>
+          <t>Pay gate conversion too low</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -9705,7 +9709,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -9715,7 +9719,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>&gt;10% refund rate</t>
+          <t>&lt;8% Draft viewers convert at 4-week mark</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -9725,7 +9729,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Forensic canvas over-delivers vs pay-gate promise; 14-day refund window</t>
+          <t>Pay-gate previews use actual canvas data; pricing differentiated by job not features; A/B test framing</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
@@ -9738,7 +9742,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Asset tracking sucks Beta scope dry</t>
+          <t>Refund rate is high</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -9758,7 +9762,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Builder spending &gt;2 weeks on asset tracking in beta phase</t>
+          <t>&gt;10% refund rate</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -9768,7 +9772,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Decision gate at end of Alpha with hard threshold; v1 only if shipped</t>
+          <t>Forensic canvas over-delivers vs pay-gate promise; 14-day refund window</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
@@ -9781,7 +9785,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>ROI testimonials don't materialise</t>
+          <t>Asset tracking sucks Beta scope dry</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -9791,7 +9795,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -9801,7 +9805,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>&lt;3 testimonials by week 4 of beta</t>
+          <t>Builder spending &gt;2 weeks on asset tracking in beta phase</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -9811,14 +9815,10 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Testimonial harvest sequence baked in from day 1; results-focused user selection</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>Kills the marketing engine if it materialises.</t>
-        </is>
-      </c>
+          <t>Decision gate at end of Alpha with hard threshold; v1 only if shipped</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr"/>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -9828,12 +9828,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>GA acquisition CAC too high</t>
+          <t>ROI testimonials don't materialise</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>Beta</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -9848,7 +9848,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Paid CAC payback &gt;4 months after 30 days of spend</t>
+          <t>&lt;3 testimonials by week 4 of beta</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -9858,10 +9858,14 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Build organic foundation in beta; don't scale paid until CAC payback known</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr"/>
+          <t>Testimonial harvest sequence baked in from day 1; results-focused user selection</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Kills the marketing engine if it materialises. Downstream symptom of R-001.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -9871,7 +9875,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Retention below unit economics floor</t>
+          <t>GA acquisition CAC too high</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -9881,7 +9885,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -9891,7 +9895,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>&lt;50% retention at week 4</t>
+          <t>Paid CAC payback &gt;4 months after 30 days of spend</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -9901,7 +9905,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Retention motion built before GA; quarterly Voice of Customer refresh designed in</t>
+          <t>Build organic foundation in beta; don't scale paid until CAC payback known</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
@@ -9914,17 +9918,17 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>TikTok algorithm de-prioritises long-form B2B content</t>
+          <t>Retention below unit economics floor</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Post-GA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -9934,7 +9938,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Organic engagement &lt;2% after 30 days of content</t>
+          <t>&lt;50% retention at week 4</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -9944,7 +9948,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Organic test before paid; cap spend at £500/wk in test phase</t>
+          <t>Retention motion built before GA; quarterly Voice of Customer refresh designed in</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr"/>
@@ -9957,12 +9961,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Trevor's bandwidth limits content production</t>
+          <t>TikTok algorithm de-prioritises long-form B2B content</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Post-GA</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -9977,7 +9981,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Trevor unavailable &gt;2 weeks consecutively</t>
+          <t>Organic engagement &lt;2% after 30 days of content</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -9987,7 +9991,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Batch recording; async content review; develop a second voice as backup</t>
+          <t>Organic test before paid; cap spend at £500/wk in test phase</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
@@ -10000,27 +10004,27 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Lovable.dev vs existing codebase architectural collision</t>
+          <t>Trevor's bandwidth limits content production</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Alpha</t>
+          <t>All</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>triggered</t>
+          <t>monitoring</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Two parallel codebases active &gt;1 week</t>
+          <t>Trevor unavailable &gt;2 weeks consecutively</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -10030,14 +10034,10 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Decide explicitly at sprint start which is canonical (F-052)</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>Status set to triggered because the decision is currently open and Gen 3 work is paused on this call.</t>
-        </is>
-      </c>
+          <t>Batch recording; async content review; develop a second voice as backup</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr"/>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -10047,27 +10047,27 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Competitor launches similar tool</t>
+          <t>Lovable.dev vs existing codebase architectural collision</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Beta</t>
+          <t>Alpha</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>monitoring</t>
+          <t>triggered</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Competitor announcement or feature ship</t>
+          <t>Two parallel codebases active &gt;1 week</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -10077,10 +10077,14 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Speed; first-mover positioning on Forensic Avatar Builder; lean into Voice of Customer differentiator</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr"/>
+          <t>Decide explicitly at sprint start which is canonical (F-052)</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Status set to triggered because the decision is currently open and Gen 3 work is paused on this call.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -10090,17 +10094,17 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Trevor changes framework spec mid-build</t>
+          <t>Competitor launches similar tool</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Beta</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -10110,7 +10114,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Any framework field change requested post-Alpha launch</t>
+          <t>Competitor announcement or feature ship</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -10120,7 +10124,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Lock the v2 Brief; require written sign-off on changes; version-tag the build</t>
+          <t>Speed; first-mover positioning on Forensic Avatar Builder; lean into Voice of Customer differentiator</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr"/>
@@ -10133,7 +10137,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Product doesn't solve enough user problems well enough to earn value</t>
+          <t>Trevor changes framework spec mid-build</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -10143,7 +10147,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -10153,7 +10157,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>At Alpha exit, fewer than 2 of {P-001, P-002, P-003} verified PARTIAL+ via tester debriefs; OR &lt;50% of testers can articulate one concrete way the canvas changed how they think about their customer; OR fewer than 60% of shipped features map to ≥1 problem.</t>
+          <t>Any framework field change requested post-Alpha launch</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -10163,14 +10167,10 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Problems sheet operationalises tracking. Alpha feedback Moments 1 + 2 measure perceived value directly. If signal is low at Alpha midpoint, narrow scope to deepen 1-2 problems rather than adding features.</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>Meta-risk above R-003 (form not conversation) and R-007 (no testimonials). The failure mode where every feature ships on time but the product still doesn't matter to anyone. Operational tool: the Problems sheet — every feature should tag to at least one problem.</t>
-        </is>
-      </c>
+          <t>Lock the v2 Brief; require written sign-off on changes; version-tag the build</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>